<commit_message>
added nodemailier, searchapi and many more changes
</commit_message>
<xml_diff>
--- a/backend/exports/history-orders-7days.xlsx
+++ b/backend/exports/history-orders-7days.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="70">
   <si>
     <t>📊 HISTORY-ORDERS REPORT</t>
   </si>
@@ -37,55 +37,190 @@
     <t>TotalAmount</t>
   </si>
   <si>
+    <t>3/6/2026</t>
+  </si>
+  <si>
+    <t>69aabaf3a3a8687782b40386</t>
+  </si>
+  <si>
+    <t>mr malik</t>
+  </si>
+  <si>
+    <t>mrmalik@gmail.com</t>
+  </si>
+  <si>
+    <t>CONFIRMED</t>
+  </si>
+  <si>
+    <t>69aab9cda3a8687782b3fed2</t>
+  </si>
+  <si>
+    <t>69aab96ea3a8687782b3fcb0</t>
+  </si>
+  <si>
+    <t>69aab8f6a3a8687782b3f8fb</t>
+  </si>
+  <si>
+    <t>69aab27137d344b575449cd2</t>
+  </si>
+  <si>
+    <t>69aaa96fdff11bc77ff8ec32</t>
+  </si>
+  <si>
+    <t>69aaa941b84907db581d3785</t>
+  </si>
+  <si>
+    <t>69aaa91be1825170c9e69cb4</t>
+  </si>
+  <si>
+    <t>69aaa7f4d7a74e6eb65d35fa</t>
+  </si>
+  <si>
+    <t>69aa623cab2d880119936f67</t>
+  </si>
+  <si>
+    <t>CANCELLED</t>
+  </si>
+  <si>
+    <t>69aa6212ab2d880119936de7</t>
+  </si>
+  <si>
+    <t>69aa60d12038c5a32ccb86cf</t>
+  </si>
+  <si>
+    <t>69aa5ebc005159cd540b9b21</t>
+  </si>
+  <si>
+    <t>69aa5e68005159cd540b99c5</t>
+  </si>
+  <si>
+    <t>3/5/2026</t>
+  </si>
+  <si>
+    <t>69a96ef90f4c9341bb4a84ce</t>
+  </si>
+  <si>
+    <t>69a96ec10f4c9341bb4a82fe</t>
+  </si>
+  <si>
+    <t>69a94ca125dcd5e4e801685d</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016866</t>
+  </si>
+  <si>
+    <t>69a92be9c3892d8ee7f43e40</t>
+  </si>
+  <si>
+    <t>69a92b8ac3892d8ee7f43da4</t>
+  </si>
+  <si>
+    <t>69a9265ac3892d8ee7f43977</t>
+  </si>
+  <si>
+    <t>69a92088928a55fe5434b7ee</t>
+  </si>
+  <si>
+    <t>69a91fed928a55fe5434b6fb</t>
+  </si>
+  <si>
+    <t>69a91f6ba468fe13be6bf990</t>
+  </si>
+  <si>
+    <t>69a91f64a468fe13be6bf97e</t>
+  </si>
+  <si>
+    <t>69a91f04a468fe13be6bf8d5</t>
+  </si>
+  <si>
+    <t>69a9188039ea7780647fe977</t>
+  </si>
+  <si>
+    <t>3/4/2026</t>
+  </si>
+  <si>
+    <t>69a94ca125dcd5e4e801685c</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016865</t>
+  </si>
+  <si>
+    <t>3/3/2026</t>
+  </si>
+  <si>
+    <t>69a6d6433440ff63a2c95390</t>
+  </si>
+  <si>
+    <t>danish</t>
+  </si>
+  <si>
+    <t>danishyt123@gmail.com</t>
+  </si>
+  <si>
+    <t>69a6d5a13440ff63a2c952c1</t>
+  </si>
+  <si>
+    <t>69a6d01248ded846f8aa1049</t>
+  </si>
+  <si>
+    <t>snow</t>
+  </si>
+  <si>
+    <t>snow@gmail.com</t>
+  </si>
+  <si>
+    <t>69a6cf05a26a0f6b958f6db8</t>
+  </si>
+  <si>
+    <t>69a6ca73bd20dddd254cded7</t>
+  </si>
+  <si>
+    <t>69a6c8103f1f952048983fae</t>
+  </si>
+  <si>
+    <t>69a94ca125dcd5e4e801685b</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016864</t>
+  </si>
+  <si>
     <t>3/2/2026</t>
   </si>
   <si>
-    <t>69a54e2d37773c078f8b4d52</t>
-  </si>
-  <si>
-    <t>snow</t>
-  </si>
-  <si>
-    <t>snow@gmail.com</t>
-  </si>
-  <si>
-    <t>CANCELLED</t>
-  </si>
-  <si>
-    <t>69a53366f12479f383972459</t>
-  </si>
-  <si>
-    <t>69a5258c291dc02602254e42</t>
-  </si>
-  <si>
-    <t>CONFIRMED</t>
+    <t>69a94ca125dcd5e4e801685a</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016863</t>
+  </si>
+  <si>
+    <t>3/1/2026</t>
+  </si>
+  <si>
+    <t>69a94ae525dcd5e4e801684d</t>
+  </si>
+  <si>
+    <t>69a94ca125dcd5e4e8016859</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016862</t>
+  </si>
+  <si>
+    <t>2/28/2026</t>
+  </si>
+  <si>
+    <t>69a94ca125dcd5e4e8016858</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016861</t>
   </si>
   <si>
     <t>2/27/2026</t>
   </si>
   <si>
-    <t>69a148625d00b578a375f304</t>
-  </si>
-  <si>
-    <t>2/26/2026</t>
-  </si>
-  <si>
-    <t>699ff1d2405f3e9d2a1d2bd9</t>
-  </si>
-  <si>
-    <t>kitty</t>
-  </si>
-  <si>
-    <t>kitty@gmail.com</t>
-  </si>
-  <si>
-    <t>699fe997405f3e9d2a1d2ae0</t>
-  </si>
-  <si>
-    <t>john</t>
-  </si>
-  <si>
-    <t>johnwick@gmail.com</t>
+    <t>69a94ca125dcd5e4e8016857</t>
+  </si>
+  <si>
+    <t>69a94d3125dcd5e4e8016860</t>
   </si>
 </sst>
 </file>
@@ -482,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="29" customWidth="1"/>
@@ -545,7 +680,7 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -565,7 +700,7 @@
         <v>12</v>
       </c>
       <c r="F6">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -582,18 +717,18 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F7">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -602,27 +737,27 @@
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F8">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F9">
         <v>30</v>
@@ -630,22 +765,822 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F14">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" t="s">
         <v>23</v>
       </c>
-      <c r="D10" t="s">
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
         <v>24</v>
       </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10">
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" t="s">
+        <v>47</v>
+      </c>
+      <c r="E34" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" t="s">
+        <v>46</v>
+      </c>
+      <c r="D35" t="s">
+        <v>47</v>
+      </c>
+      <c r="E35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D36" t="s">
+        <v>51</v>
+      </c>
+      <c r="E36" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" t="s">
+        <v>50</v>
+      </c>
+      <c r="D37" t="s">
+        <v>51</v>
+      </c>
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" t="s">
+        <v>53</v>
+      </c>
+      <c r="C38" t="s">
+        <v>50</v>
+      </c>
+      <c r="D38" t="s">
+        <v>51</v>
+      </c>
+      <c r="E38" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" t="s">
+        <v>54</v>
+      </c>
+      <c r="C39" t="s">
+        <v>50</v>
+      </c>
+      <c r="D39" t="s">
+        <v>51</v>
+      </c>
+      <c r="E39" t="s">
+        <v>22</v>
+      </c>
+      <c r="F39">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>44</v>
+      </c>
+      <c r="B40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C40" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40">
         <v>90</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" t="s">
+        <v>56</v>
+      </c>
+      <c r="C41" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>57</v>
+      </c>
+      <c r="B43" t="s">
+        <v>59</v>
+      </c>
+      <c r="C43" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>12</v>
+      </c>
+      <c r="F43">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>12</v>
+      </c>
+      <c r="F44">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>60</v>
+      </c>
+      <c r="B45" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" t="s">
+        <v>10</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" t="s">
+        <v>10</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" t="s">
+        <v>65</v>
+      </c>
+      <c r="C47" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" t="s">
+        <v>66</v>
+      </c>
+      <c r="C48" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>12</v>
+      </c>
+      <c r="F48">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>67</v>
+      </c>
+      <c r="B49" t="s">
+        <v>68</v>
+      </c>
+      <c r="C49" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>12</v>
+      </c>
+      <c r="F49">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50" t="s">
+        <v>69</v>
+      </c>
+      <c r="C50" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>